<commit_message>
data: seed demo fixtures for remaining detectors (plate, shared OSR, tamper, weights, prior-year); scope note in CLAUDE.md
</commit_message>
<xml_diff>
--- a/fixtures/demo/demo_exporter_AL.xlsx
+++ b/fixtures/demo/demo_exporter_AL.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R53"/>
+  <dimension ref="A1:V53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,60 +454,80 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>GROSS_WEIGHT</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>TARE_WEIGHT</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>PALLET_WEIGHT</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>WEIGHT_OF_NON_TARGET_MATERIALS</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>NET_WEIGHT</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>RECYCLABLE_PROPORTION_PERCENTAGE</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>TONNAGE_RECEIVED_FOR_EXPORT</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>TONNAGE_OF_UK_PACKAGING_WASTE_EXPORTED</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>TONNAGE_RECEIVED_BY_OSR</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>TONNAGE_PASSED_INTERIM_SITE_RECEIVED_BY_OSR</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>OSR_COUNTRY</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>OSR_NAME</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>WAS_THE_WASTE_REFUSED</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>SUPPLIER_NAME</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>SUPPLIER_POSTCODE</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>CARRIER_VEHICLE_REGISTRATION_NUMBER</t>
         </is>
@@ -516,7 +536,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>(human header)</t>
+          <t>(human)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -536,6 +556,10 @@
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -560,6 +584,10 @@
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -585,49 +613,61 @@
         </is>
       </c>
       <c r="G4" t="n">
+        <v>65</v>
+      </c>
+      <c r="H4" t="n">
+        <v>10</v>
+      </c>
+      <c r="I4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K4" t="n">
         <v>50</v>
       </c>
-      <c r="H4" t="n">
+      <c r="L4" t="n">
         <v>0.975</v>
       </c>
-      <c r="I4" t="n">
+      <c r="M4" t="n">
         <v>43.875</v>
       </c>
-      <c r="J4" t="n">
+      <c r="N4" t="n">
         <v>39.488</v>
       </c>
-      <c r="K4" t="n">
+      <c r="O4" t="n">
         <v>27.642</v>
       </c>
-      <c r="L4" t="n">
+      <c r="P4" t="n">
         <v>31.59</v>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>Germany-DE</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 0</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-0</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>AL00 0AA</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>AL00REG</t>
         </is>
@@ -657,51 +697,63 @@
         </is>
       </c>
       <c r="G5" t="n">
+        <v>72</v>
+      </c>
+      <c r="H5" t="n">
+        <v>10</v>
+      </c>
+      <c r="I5" t="n">
+        <v>5</v>
+      </c>
+      <c r="J5" t="n">
+        <v>5</v>
+      </c>
+      <c r="K5" t="n">
         <v>57</v>
       </c>
-      <c r="H5" t="n">
+      <c r="L5" t="n">
         <v>0.875</v>
       </c>
-      <c r="I5" t="n">
+      <c r="M5" t="n">
         <v>44.888</v>
       </c>
-      <c r="J5" t="n">
+      <c r="N5" t="n">
         <v>40.848</v>
       </c>
-      <c r="K5" t="n">
+      <c r="O5" t="n">
         <v>28.594</v>
       </c>
-      <c r="L5" t="n">
+      <c r="P5" t="n">
         <v>32.678</v>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>Spain-ES</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="R5" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 1</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="S5" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="T5" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-1</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>AL01 0AA</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>AL01REG</t>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>AL11REG</t>
         </is>
       </c>
     </row>
@@ -729,48 +781,60 @@
         </is>
       </c>
       <c r="G6" t="n">
+        <v>79</v>
+      </c>
+      <c r="H6" t="n">
+        <v>10</v>
+      </c>
+      <c r="I6" t="n">
+        <v>5</v>
+      </c>
+      <c r="J6" t="n">
+        <v>5</v>
+      </c>
+      <c r="K6" t="n">
         <v>64</v>
       </c>
-      <c r="H6" t="n">
+      <c r="L6" t="n">
         <v>0.65</v>
       </c>
-      <c r="I6" t="n">
+      <c r="M6" t="n">
         <v>37.44</v>
       </c>
-      <c r="J6" t="n">
+      <c r="N6" t="n">
         <v>34.445</v>
       </c>
-      <c r="K6" t="n">
+      <c r="O6" t="n">
         <v>33.067</v>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>Netherlands-NL</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="R6" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 2</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="S6" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="T6" t="inlineStr">
         <is>
           <t>Shared Metals Recovery Ltd</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>LS1 4AB</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>AL02REG</t>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>AL22REG</t>
         </is>
       </c>
     </row>
@@ -798,48 +862,60 @@
         </is>
       </c>
       <c r="G7" t="n">
+        <v>86</v>
+      </c>
+      <c r="H7" t="n">
+        <v>10</v>
+      </c>
+      <c r="I7" t="n">
+        <v>5</v>
+      </c>
+      <c r="J7" t="n">
+        <v>5</v>
+      </c>
+      <c r="K7" t="n">
         <v>71</v>
       </c>
-      <c r="H7" t="n">
+      <c r="L7" t="n">
         <v>0.975</v>
       </c>
-      <c r="I7" t="n">
+      <c r="M7" t="n">
         <v>62.302</v>
       </c>
-      <c r="J7" t="n">
+      <c r="N7" t="n">
         <v>57.941</v>
       </c>
-      <c r="K7" t="n">
+      <c r="O7" t="n">
         <v>56.782</v>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="Q7" t="inlineStr">
         <is>
           <t>India-IN</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="R7" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 3</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="S7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
+      <c r="T7" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-3</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr">
+      <c r="U7" t="inlineStr">
         <is>
           <t>AL03 0AA</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>AL03REG</t>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>AL33REG</t>
         </is>
       </c>
     </row>
@@ -867,48 +943,60 @@
         </is>
       </c>
       <c r="G8" t="n">
+        <v>93</v>
+      </c>
+      <c r="H8" t="n">
+        <v>10</v>
+      </c>
+      <c r="I8" t="n">
+        <v>5</v>
+      </c>
+      <c r="J8" t="n">
+        <v>5</v>
+      </c>
+      <c r="K8" t="n">
         <v>78</v>
       </c>
-      <c r="H8" t="n">
+      <c r="L8" t="n">
         <v>0.875</v>
       </c>
-      <c r="I8" t="n">
+      <c r="M8" t="n">
         <v>61.425</v>
       </c>
-      <c r="J8" t="n">
+      <c r="N8" t="n">
         <v>57.739</v>
       </c>
-      <c r="K8" t="n">
+      <c r="O8" t="n">
         <v>53.12</v>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="Q8" t="inlineStr">
         <is>
           <t>Turkey-TR</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="R8" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 4</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="S8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
+      <c r="T8" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-4</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr">
+      <c r="U8" t="inlineStr">
         <is>
           <t>AL04 0AA</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>AL04REG</t>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>AL44REG</t>
         </is>
       </c>
     </row>
@@ -936,51 +1024,63 @@
         </is>
       </c>
       <c r="G9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H9" t="n">
+        <v>10</v>
+      </c>
+      <c r="I9" t="n">
+        <v>5</v>
+      </c>
+      <c r="J9" t="n">
+        <v>5</v>
+      </c>
+      <c r="K9" t="n">
         <v>85</v>
       </c>
-      <c r="H9" t="n">
+      <c r="L9" t="n">
         <v>0.65</v>
       </c>
-      <c r="I9" t="n">
+      <c r="M9" t="n">
         <v>49.725</v>
       </c>
-      <c r="J9" t="n">
+      <c r="N9" t="n">
         <v>64.642</v>
       </c>
-      <c r="K9" t="n">
+      <c r="O9" t="n">
         <v>31.327</v>
       </c>
-      <c r="L9" t="n">
+      <c r="P9" t="n">
         <v>35.802</v>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="Q9" t="inlineStr">
         <is>
           <t>South Korea-KR</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="R9" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 5</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="S9" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
+      <c r="T9" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-5</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr">
+      <c r="U9" t="inlineStr">
         <is>
           <t>AL05 0AA</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>AL05REG</t>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>AL55REG</t>
         </is>
       </c>
     </row>
@@ -1008,51 +1108,63 @@
         </is>
       </c>
       <c r="G10" t="n">
+        <v>107</v>
+      </c>
+      <c r="H10" t="n">
+        <v>10</v>
+      </c>
+      <c r="I10" t="n">
+        <v>5</v>
+      </c>
+      <c r="J10" t="n">
+        <v>5</v>
+      </c>
+      <c r="K10" t="n">
         <v>92</v>
       </c>
-      <c r="H10" t="n">
+      <c r="L10" t="n">
         <v>0.975</v>
       </c>
-      <c r="I10" t="n">
+      <c r="M10" t="n">
         <v>80.73</v>
       </c>
-      <c r="J10" t="n">
+      <c r="N10" t="n">
         <v>73.464</v>
       </c>
-      <c r="K10" t="n">
+      <c r="O10" t="n">
         <v>51.425</v>
       </c>
-      <c r="L10" t="n">
+      <c r="P10" t="n">
         <v>58.771</v>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="Q10" t="inlineStr">
         <is>
           <t>Italy-IT</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="R10" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 6</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="S10" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
+      <c r="T10" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-6</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr">
+      <c r="U10" t="inlineStr">
         <is>
           <t>AL06 0AA</t>
         </is>
       </c>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>AL06REG</t>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>AL66REG</t>
         </is>
       </c>
     </row>
@@ -1080,48 +1192,60 @@
         </is>
       </c>
       <c r="G11" t="n">
+        <v>114</v>
+      </c>
+      <c r="H11" t="n">
+        <v>10</v>
+      </c>
+      <c r="I11" t="n">
+        <v>5</v>
+      </c>
+      <c r="J11" t="n">
+        <v>5</v>
+      </c>
+      <c r="K11" t="n">
         <v>99</v>
       </c>
-      <c r="H11" t="n">
+      <c r="L11" t="n">
         <v>0.35</v>
       </c>
-      <c r="I11" t="n">
+      <c r="M11" t="n">
         <v>77.96299999999999</v>
       </c>
-      <c r="J11" t="n">
+      <c r="N11" t="n">
         <v>71.726</v>
       </c>
-      <c r="K11" t="n">
+      <c r="O11" t="n">
         <v>70.291</v>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="Q11" t="inlineStr">
         <is>
           <t>Germany-DE</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="R11" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 7</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
+      <c r="S11" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
+      <c r="T11" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-7</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr">
+      <c r="U11" t="inlineStr">
         <is>
           <t>AL07 0AA</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>AL07REG</t>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>AL77REG</t>
         </is>
       </c>
     </row>
@@ -1149,48 +1273,60 @@
         </is>
       </c>
       <c r="G12" t="n">
+        <v>121</v>
+      </c>
+      <c r="H12" t="n">
+        <v>10</v>
+      </c>
+      <c r="I12" t="n">
+        <v>5</v>
+      </c>
+      <c r="J12" t="n">
+        <v>5</v>
+      </c>
+      <c r="K12" t="n">
         <v>106</v>
       </c>
-      <c r="H12" t="n">
+      <c r="L12" t="n">
         <v>0.65</v>
       </c>
-      <c r="I12" t="n">
+      <c r="M12" t="n">
         <v>62.01</v>
       </c>
-      <c r="J12" t="n">
+      <c r="N12" t="n">
         <v>57.669</v>
       </c>
-      <c r="K12" t="n">
+      <c r="O12" t="n">
         <v>80.73699999999999</v>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="Q12" t="inlineStr">
         <is>
           <t>Spain-ES</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
+      <c r="R12" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 8</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr">
+      <c r="S12" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr">
+      <c r="T12" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-8</t>
         </is>
       </c>
-      <c r="Q12" t="inlineStr">
+      <c r="U12" t="inlineStr">
         <is>
           <t>AL08 0AA</t>
         </is>
       </c>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t>AL08REG</t>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>AL88REG</t>
         </is>
       </c>
     </row>
@@ -1218,48 +1354,60 @@
         </is>
       </c>
       <c r="G13" t="n">
+        <v>128</v>
+      </c>
+      <c r="H13" t="n">
+        <v>10</v>
+      </c>
+      <c r="I13" t="n">
+        <v>5</v>
+      </c>
+      <c r="J13" t="n">
+        <v>5</v>
+      </c>
+      <c r="K13" t="n">
         <v>113</v>
       </c>
-      <c r="H13" t="n">
+      <c r="L13" t="n">
         <v>0.975</v>
       </c>
-      <c r="I13" t="n">
+      <c r="M13" t="n">
         <v>99.157</v>
       </c>
-      <c r="J13" t="n">
+      <c r="N13" t="n">
         <v>93.208</v>
       </c>
-      <c r="K13" t="n">
+      <c r="O13" t="n">
         <v>87.616</v>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="Q13" t="inlineStr">
         <is>
           <t>Tuvalu-TV</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
+      <c r="R13" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 9</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr">
+      <c r="S13" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr">
+      <c r="T13" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-9</t>
         </is>
       </c>
-      <c r="Q13" t="inlineStr">
+      <c r="U13" t="inlineStr">
         <is>
           <t>AL09 0AA</t>
         </is>
       </c>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>AL09REG</t>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>AL99REG</t>
         </is>
       </c>
     </row>
@@ -1287,51 +1435,63 @@
         </is>
       </c>
       <c r="G14" t="n">
+        <v>135</v>
+      </c>
+      <c r="H14" t="n">
+        <v>10</v>
+      </c>
+      <c r="I14" t="n">
+        <v>5</v>
+      </c>
+      <c r="J14" t="n">
+        <v>5</v>
+      </c>
+      <c r="K14" t="n">
         <v>120</v>
       </c>
-      <c r="H14" t="n">
+      <c r="L14" t="n">
         <v>0.875</v>
       </c>
-      <c r="I14" t="n">
+      <c r="M14" t="n">
         <v>94.5</v>
       </c>
-      <c r="J14" t="n">
+      <c r="N14" t="n">
         <v>85.05</v>
       </c>
-      <c r="K14" t="n">
+      <c r="O14" t="n">
         <v>59.535</v>
       </c>
-      <c r="L14" t="n">
+      <c r="P14" t="n">
         <v>68.04000000000001</v>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="Q14" t="inlineStr">
         <is>
           <t>India-IN</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr">
+      <c r="R14" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 10</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr">
+      <c r="S14" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr">
+      <c r="T14" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-10</t>
         </is>
       </c>
-      <c r="Q14" t="inlineStr">
+      <c r="U14" t="inlineStr">
         <is>
           <t>AL10 0AA</t>
         </is>
       </c>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>AL10REG</t>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>AL00REG</t>
         </is>
       </c>
     </row>
@@ -1359,49 +1519,61 @@
         </is>
       </c>
       <c r="G15" t="n">
+        <v>142</v>
+      </c>
+      <c r="H15" t="n">
+        <v>10</v>
+      </c>
+      <c r="I15" t="n">
+        <v>5</v>
+      </c>
+      <c r="J15" t="n">
+        <v>5</v>
+      </c>
+      <c r="K15" t="n">
         <v>127</v>
       </c>
-      <c r="H15" t="n">
+      <c r="L15" t="n">
         <v>0.65</v>
       </c>
-      <c r="I15" t="n">
+      <c r="M15" t="n">
         <v>74.295</v>
       </c>
-      <c r="J15" t="n">
+      <c r="N15" t="n">
         <v>67.608</v>
       </c>
-      <c r="K15" t="n">
+      <c r="O15" t="n">
         <v>47.326</v>
       </c>
-      <c r="L15" t="n">
+      <c r="P15" t="n">
         <v>54.086</v>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="Q15" t="inlineStr">
         <is>
           <t>Turkey-TR</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr">
+      <c r="R15" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 11</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr">
+      <c r="S15" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr">
+      <c r="T15" t="inlineStr">
         <is>
           <t>Shared Metals Recovery Ltd</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr">
+      <c r="U15" t="inlineStr">
         <is>
           <t>LS1 4AB</t>
         </is>
       </c>
-      <c r="R15" t="inlineStr">
+      <c r="V15" t="inlineStr">
         <is>
           <t>AL11REG</t>
         </is>
@@ -1431,48 +1603,60 @@
         </is>
       </c>
       <c r="G16" t="n">
+        <v>149</v>
+      </c>
+      <c r="H16" t="n">
+        <v>10</v>
+      </c>
+      <c r="I16" t="n">
+        <v>5</v>
+      </c>
+      <c r="J16" t="n">
+        <v>5</v>
+      </c>
+      <c r="K16" t="n">
         <v>134</v>
       </c>
-      <c r="H16" t="n">
+      <c r="L16" t="n">
         <v>0.975</v>
       </c>
-      <c r="I16" t="n">
+      <c r="M16" t="n">
         <v>117.585</v>
       </c>
-      <c r="J16" t="n">
+      <c r="N16" t="n">
         <v>108.178</v>
       </c>
-      <c r="K16" t="n">
+      <c r="O16" t="n">
         <v>99.524</v>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="Q16" t="inlineStr">
         <is>
           <t>South Korea-KR</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr">
+      <c r="R16" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 12</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr">
+      <c r="S16" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr">
+      <c r="T16" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-12</t>
         </is>
       </c>
-      <c r="Q16" t="inlineStr">
+      <c r="U16" t="inlineStr">
         <is>
           <t>AL12 0AA</t>
         </is>
       </c>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>AL12REG</t>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>AL22REG</t>
         </is>
       </c>
     </row>
@@ -1500,46 +1684,58 @@
         </is>
       </c>
       <c r="G17" t="n">
+        <v>156</v>
+      </c>
+      <c r="H17" t="n">
+        <v>10</v>
+      </c>
+      <c r="I17" t="n">
+        <v>5</v>
+      </c>
+      <c r="J17" t="n">
+        <v>5</v>
+      </c>
+      <c r="K17" t="n">
         <v>141</v>
       </c>
-      <c r="H17" t="n">
+      <c r="L17" t="n">
         <v>0.875</v>
       </c>
-      <c r="I17" t="n">
+      <c r="M17" t="n">
         <v>111.038</v>
       </c>
-      <c r="J17" t="n">
+      <c r="N17" t="n">
         <v>103.265</v>
       </c>
-      <c r="K17" t="n">
+      <c r="O17" t="n">
         <v>97.069</v>
       </c>
-      <c r="M17" t="inlineStr">
+      <c r="Q17" t="inlineStr">
         <is>
           <t>Italy-IT</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr">
+      <c r="R17" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 13</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr">
+      <c r="S17" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr">
+      <c r="T17" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-13</t>
         </is>
       </c>
-      <c r="Q17" t="inlineStr">
+      <c r="U17" t="inlineStr">
         <is>
           <t>AL13 0AA</t>
         </is>
       </c>
-      <c r="R17" t="inlineStr">
+      <c r="V17" t="inlineStr">
         <is>
           <t>SH24RED</t>
         </is>
@@ -1569,48 +1765,60 @@
         </is>
       </c>
       <c r="G18" t="n">
+        <v>163</v>
+      </c>
+      <c r="H18" t="n">
+        <v>10</v>
+      </c>
+      <c r="I18" t="n">
+        <v>5</v>
+      </c>
+      <c r="J18" t="n">
+        <v>5</v>
+      </c>
+      <c r="K18" t="n">
         <v>148</v>
       </c>
-      <c r="H18" t="n">
+      <c r="L18" t="n">
         <v>0.65</v>
       </c>
-      <c r="I18" t="n">
+      <c r="M18" t="n">
         <v>86.58</v>
       </c>
-      <c r="J18" t="n">
+      <c r="N18" t="n">
         <v>81.38500000000001</v>
       </c>
-      <c r="K18" t="n">
+      <c r="O18" t="n">
         <v>78.13</v>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="Q18" t="inlineStr">
         <is>
           <t>Germany-DE</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr">
+      <c r="R18" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 14</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr">
+      <c r="S18" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr">
+      <c r="T18" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-14</t>
         </is>
       </c>
-      <c r="Q18" t="inlineStr">
+      <c r="U18" t="inlineStr">
         <is>
           <t>AL14 0AA</t>
         </is>
       </c>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>AL14REG</t>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>AL44REG</t>
         </is>
       </c>
     </row>
@@ -1638,51 +1846,63 @@
         </is>
       </c>
       <c r="G19" t="n">
+        <v>170</v>
+      </c>
+      <c r="H19" t="n">
+        <v>10</v>
+      </c>
+      <c r="I19" t="n">
+        <v>5</v>
+      </c>
+      <c r="J19" t="n">
+        <v>5</v>
+      </c>
+      <c r="K19" t="n">
         <v>155</v>
       </c>
-      <c r="H19" t="n">
+      <c r="L19" t="n">
         <v>0.975</v>
       </c>
-      <c r="I19" t="n">
+      <c r="M19" t="n">
         <v>136.013</v>
       </c>
-      <c r="J19" t="n">
+      <c r="N19" t="n">
         <v>176.817</v>
       </c>
-      <c r="K19" t="n">
+      <c r="O19" t="n">
         <v>85.688</v>
       </c>
-      <c r="L19" t="n">
+      <c r="P19" t="n">
         <v>97.93000000000001</v>
       </c>
-      <c r="M19" t="inlineStr">
+      <c r="Q19" t="inlineStr">
         <is>
           <t>Spain-ES</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr">
+      <c r="R19" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 15</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr">
+      <c r="S19" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr">
+      <c r="T19" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-15</t>
         </is>
       </c>
-      <c r="Q19" t="inlineStr">
+      <c r="U19" t="inlineStr">
         <is>
           <t>AL15 0AA</t>
         </is>
       </c>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>AL15REG</t>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>AL55REG</t>
         </is>
       </c>
     </row>
@@ -1710,51 +1930,63 @@
         </is>
       </c>
       <c r="G20" t="n">
+        <v>177</v>
+      </c>
+      <c r="H20" t="n">
+        <v>10</v>
+      </c>
+      <c r="I20" t="n">
+        <v>5</v>
+      </c>
+      <c r="J20" t="n">
+        <v>5</v>
+      </c>
+      <c r="K20" t="n">
         <v>162</v>
       </c>
-      <c r="H20" t="n">
+      <c r="L20" t="n">
         <v>0.875</v>
       </c>
-      <c r="I20" t="n">
+      <c r="M20" t="n">
         <v>127.575</v>
       </c>
-      <c r="J20" t="n">
+      <c r="N20" t="n">
         <v>116.093</v>
       </c>
-      <c r="K20" t="n">
+      <c r="O20" t="n">
         <v>81.265</v>
       </c>
-      <c r="L20" t="n">
+      <c r="P20" t="n">
         <v>92.874</v>
       </c>
-      <c r="M20" t="inlineStr">
+      <c r="Q20" t="inlineStr">
         <is>
           <t>Netherlands-NL</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr">
+      <c r="R20" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 16</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr">
+      <c r="S20" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr">
+      <c r="T20" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-16</t>
         </is>
       </c>
-      <c r="Q20" t="inlineStr">
+      <c r="U20" t="inlineStr">
         <is>
           <t>AL16 0AA</t>
         </is>
       </c>
-      <c r="R20" t="inlineStr">
-        <is>
-          <t>AL16REG</t>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>AL66REG</t>
         </is>
       </c>
     </row>
@@ -1782,48 +2014,60 @@
         </is>
       </c>
       <c r="G21" t="n">
+        <v>184</v>
+      </c>
+      <c r="H21" t="n">
+        <v>10</v>
+      </c>
+      <c r="I21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J21" t="n">
+        <v>5</v>
+      </c>
+      <c r="K21" t="n">
         <v>169</v>
       </c>
-      <c r="H21" t="n">
+      <c r="L21" t="n">
         <v>0.35</v>
       </c>
-      <c r="I21" t="n">
+      <c r="M21" t="n">
         <v>98.86499999999999</v>
       </c>
-      <c r="J21" t="n">
+      <c r="N21" t="n">
         <v>90.956</v>
       </c>
-      <c r="K21" t="n">
+      <c r="O21" t="n">
         <v>85.499</v>
       </c>
-      <c r="M21" t="inlineStr">
+      <c r="Q21" t="inlineStr">
         <is>
           <t>India-IN</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr">
+      <c r="R21" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 17</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr">
+      <c r="S21" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr">
+      <c r="T21" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-17</t>
         </is>
       </c>
-      <c r="Q21" t="inlineStr">
+      <c r="U21" t="inlineStr">
         <is>
           <t>AL17 0AA</t>
         </is>
       </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>AL17REG</t>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>AL77REG</t>
         </is>
       </c>
     </row>
@@ -1851,48 +2095,60 @@
         </is>
       </c>
       <c r="G22" t="n">
+        <v>191</v>
+      </c>
+      <c r="H22" t="n">
+        <v>10</v>
+      </c>
+      <c r="I22" t="n">
+        <v>5</v>
+      </c>
+      <c r="J22" t="n">
+        <v>5</v>
+      </c>
+      <c r="K22" t="n">
         <v>176</v>
       </c>
-      <c r="H22" t="n">
+      <c r="L22" t="n">
         <v>0.975</v>
       </c>
-      <c r="I22" t="n">
+      <c r="M22" t="n">
         <v>154.44</v>
       </c>
-      <c r="J22" t="n">
+      <c r="N22" t="n">
         <v>143.629</v>
       </c>
-      <c r="K22" t="n">
+      <c r="O22" t="n">
         <v>201.081</v>
       </c>
-      <c r="M22" t="inlineStr">
+      <c r="Q22" t="inlineStr">
         <is>
           <t>Turkey-TR</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr">
+      <c r="R22" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 18</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr">
+      <c r="S22" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr">
+      <c r="T22" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-18</t>
         </is>
       </c>
-      <c r="Q22" t="inlineStr">
+      <c r="U22" t="inlineStr">
         <is>
           <t>AL18 0AA</t>
         </is>
       </c>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>AL18REG</t>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>AL88REG</t>
         </is>
       </c>
     </row>
@@ -1920,48 +2176,60 @@
         </is>
       </c>
       <c r="G23" t="n">
+        <v>198</v>
+      </c>
+      <c r="H23" t="n">
+        <v>10</v>
+      </c>
+      <c r="I23" t="n">
+        <v>5</v>
+      </c>
+      <c r="J23" t="n">
+        <v>5</v>
+      </c>
+      <c r="K23" t="n">
         <v>183</v>
       </c>
-      <c r="H23" t="n">
+      <c r="L23" t="n">
         <v>0.875</v>
       </c>
-      <c r="I23" t="n">
+      <c r="M23" t="n">
         <v>144.113</v>
       </c>
-      <c r="J23" t="n">
+      <c r="N23" t="n">
         <v>135.466</v>
       </c>
-      <c r="K23" t="n">
+      <c r="O23" t="n">
         <v>132.757</v>
       </c>
-      <c r="M23" t="inlineStr">
+      <c r="Q23" t="inlineStr">
         <is>
           <t>Nauru-NR</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr">
+      <c r="R23" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 19</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr">
+      <c r="S23" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr">
+      <c r="T23" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-19</t>
         </is>
       </c>
-      <c r="Q23" t="inlineStr">
+      <c r="U23" t="inlineStr">
         <is>
           <t>AL19 0AA</t>
         </is>
       </c>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t>AL19REG</t>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>AL99REG</t>
         </is>
       </c>
     </row>
@@ -1989,51 +2257,63 @@
         </is>
       </c>
       <c r="G24" t="n">
+        <v>205</v>
+      </c>
+      <c r="H24" t="n">
+        <v>10</v>
+      </c>
+      <c r="I24" t="n">
+        <v>5</v>
+      </c>
+      <c r="J24" t="n">
+        <v>5</v>
+      </c>
+      <c r="K24" t="n">
         <v>190</v>
       </c>
-      <c r="H24" t="n">
+      <c r="L24" t="n">
         <v>0.65</v>
       </c>
-      <c r="I24" t="n">
+      <c r="M24" t="n">
         <v>111.15</v>
       </c>
-      <c r="J24" t="n">
+      <c r="N24" t="n">
         <v>100.035</v>
       </c>
-      <c r="K24" t="n">
+      <c r="O24" t="n">
         <v>70.024</v>
       </c>
-      <c r="L24" t="n">
+      <c r="P24" t="n">
         <v>80.02800000000001</v>
       </c>
-      <c r="M24" t="inlineStr">
+      <c r="Q24" t="inlineStr">
         <is>
           <t>Italy-IT</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr">
+      <c r="R24" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 20</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr">
+      <c r="S24" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P24" t="inlineStr">
+      <c r="T24" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-20</t>
         </is>
       </c>
-      <c r="Q24" t="inlineStr">
+      <c r="U24" t="inlineStr">
         <is>
           <t>AL20 0AA</t>
         </is>
       </c>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t>AL20REG</t>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>AL00REG</t>
         </is>
       </c>
     </row>
@@ -2061,51 +2341,63 @@
         </is>
       </c>
       <c r="G25" t="n">
+        <v>212</v>
+      </c>
+      <c r="H25" t="n">
+        <v>10</v>
+      </c>
+      <c r="I25" t="n">
+        <v>5</v>
+      </c>
+      <c r="J25" t="n">
+        <v>5</v>
+      </c>
+      <c r="K25" t="n">
         <v>197</v>
       </c>
-      <c r="H25" t="n">
+      <c r="L25" t="n">
         <v>0.975</v>
       </c>
-      <c r="I25" t="n">
+      <c r="M25" t="n">
         <v>172.868</v>
       </c>
-      <c r="J25" t="n">
+      <c r="N25" t="n">
         <v>157.31</v>
       </c>
-      <c r="K25" t="n">
+      <c r="O25" t="n">
         <v>110.117</v>
       </c>
-      <c r="L25" t="n">
+      <c r="P25" t="n">
         <v>125.848</v>
       </c>
-      <c r="M25" t="inlineStr">
+      <c r="Q25" t="inlineStr">
         <is>
           <t>Germany-DE</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr">
+      <c r="R25" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 21</t>
         </is>
       </c>
-      <c r="O25" t="inlineStr">
+      <c r="S25" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P25" t="inlineStr">
+      <c r="T25" t="inlineStr">
         <is>
           <t>Shared Metals Recovery Ltd</t>
         </is>
       </c>
-      <c r="Q25" t="inlineStr">
+      <c r="U25" t="inlineStr">
         <is>
           <t>LS1 4AB</t>
         </is>
       </c>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>AL21REG</t>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>AL11REG</t>
         </is>
       </c>
     </row>
@@ -2133,46 +2425,58 @@
         </is>
       </c>
       <c r="G26" t="n">
+        <v>219</v>
+      </c>
+      <c r="H26" t="n">
+        <v>10</v>
+      </c>
+      <c r="I26" t="n">
+        <v>5</v>
+      </c>
+      <c r="J26" t="n">
+        <v>5</v>
+      </c>
+      <c r="K26" t="n">
         <v>204</v>
       </c>
-      <c r="H26" t="n">
+      <c r="L26" t="n">
         <v>0.875</v>
       </c>
-      <c r="I26" t="n">
+      <c r="M26" t="n">
         <v>160.65</v>
       </c>
-      <c r="J26" t="n">
+      <c r="N26" t="n">
         <v>147.798</v>
       </c>
-      <c r="K26" t="n">
+      <c r="O26" t="n">
         <v>141.886</v>
       </c>
-      <c r="M26" t="inlineStr">
+      <c r="Q26" t="inlineStr">
         <is>
           <t>Spain-ES</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr">
+      <c r="R26" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 22</t>
         </is>
       </c>
-      <c r="O26" t="inlineStr">
+      <c r="S26" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr">
+      <c r="T26" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-22</t>
         </is>
       </c>
-      <c r="Q26" t="inlineStr">
+      <c r="U26" t="inlineStr">
         <is>
           <t>AL22 0AA</t>
         </is>
       </c>
-      <c r="R26" t="inlineStr">
+      <c r="V26" t="inlineStr">
         <is>
           <t>AL22REG</t>
         </is>
@@ -2202,46 +2506,58 @@
         </is>
       </c>
       <c r="G27" t="n">
+        <v>226</v>
+      </c>
+      <c r="H27" t="n">
+        <v>10</v>
+      </c>
+      <c r="I27" t="n">
+        <v>5</v>
+      </c>
+      <c r="J27" t="n">
+        <v>5</v>
+      </c>
+      <c r="K27" t="n">
         <v>211</v>
       </c>
-      <c r="H27" t="n">
+      <c r="L27" t="n">
         <v>0.65</v>
       </c>
-      <c r="I27" t="n">
+      <c r="M27" t="n">
         <v>123.435</v>
       </c>
-      <c r="J27" t="n">
+      <c r="N27" t="n">
         <v>114.795</v>
       </c>
-      <c r="K27" t="n">
+      <c r="O27" t="n">
         <v>112.499</v>
       </c>
-      <c r="M27" t="inlineStr">
+      <c r="Q27" t="inlineStr">
         <is>
           <t>Netherlands-NL</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr">
+      <c r="R27" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 23</t>
         </is>
       </c>
-      <c r="O27" t="inlineStr">
+      <c r="S27" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr">
+      <c r="T27" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-23</t>
         </is>
       </c>
-      <c r="Q27" t="inlineStr">
+      <c r="U27" t="inlineStr">
         <is>
           <t>AL23 0AA</t>
         </is>
       </c>
-      <c r="R27" t="inlineStr">
+      <c r="V27" t="inlineStr">
         <is>
           <t>SH24RED</t>
         </is>
@@ -2271,48 +2587,60 @@
         </is>
       </c>
       <c r="G28" t="n">
+        <v>233</v>
+      </c>
+      <c r="H28" t="n">
+        <v>10</v>
+      </c>
+      <c r="I28" t="n">
+        <v>5</v>
+      </c>
+      <c r="J28" t="n">
+        <v>5</v>
+      </c>
+      <c r="K28" t="n">
         <v>218</v>
       </c>
-      <c r="H28" t="n">
+      <c r="L28" t="n">
         <v>0.975</v>
       </c>
-      <c r="I28" t="n">
+      <c r="M28" t="n">
         <v>191.295</v>
       </c>
-      <c r="J28" t="n">
+      <c r="N28" t="n">
         <v>179.817</v>
       </c>
-      <c r="K28" t="n">
+      <c r="O28" t="n">
         <v>165.432</v>
       </c>
-      <c r="M28" t="inlineStr">
+      <c r="Q28" t="inlineStr">
         <is>
           <t>India-IN</t>
         </is>
       </c>
-      <c r="N28" t="inlineStr">
+      <c r="R28" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 24</t>
         </is>
       </c>
-      <c r="O28" t="inlineStr">
+      <c r="S28" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P28" t="inlineStr">
+      <c r="T28" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-24</t>
         </is>
       </c>
-      <c r="Q28" t="inlineStr">
+      <c r="U28" t="inlineStr">
         <is>
           <t>AL24 0AA</t>
         </is>
       </c>
-      <c r="R28" t="inlineStr">
-        <is>
-          <t>AL24REG</t>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>AL44REG</t>
         </is>
       </c>
     </row>
@@ -2340,51 +2668,63 @@
         </is>
       </c>
       <c r="G29" t="n">
+        <v>240</v>
+      </c>
+      <c r="H29" t="n">
+        <v>10</v>
+      </c>
+      <c r="I29" t="n">
+        <v>5</v>
+      </c>
+      <c r="J29" t="n">
+        <v>5</v>
+      </c>
+      <c r="K29" t="n">
         <v>225</v>
       </c>
-      <c r="H29" t="n">
+      <c r="L29" t="n">
         <v>0.875</v>
       </c>
-      <c r="I29" t="n">
+      <c r="M29" t="n">
         <v>177.188</v>
       </c>
-      <c r="J29" t="n">
+      <c r="N29" t="n">
         <v>230.344</v>
       </c>
-      <c r="K29" t="n">
+      <c r="O29" t="n">
         <v>111.628</v>
       </c>
-      <c r="L29" t="n">
+      <c r="P29" t="n">
         <v>127.575</v>
       </c>
-      <c r="M29" t="inlineStr">
+      <c r="Q29" t="inlineStr">
         <is>
           <t>Turkey-TR</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr">
+      <c r="R29" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 25</t>
         </is>
       </c>
-      <c r="O29" t="inlineStr">
+      <c r="S29" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P29" t="inlineStr">
+      <c r="T29" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-25</t>
         </is>
       </c>
-      <c r="Q29" t="inlineStr">
+      <c r="U29" t="inlineStr">
         <is>
           <t>AL25 0AA</t>
         </is>
       </c>
-      <c r="R29" t="inlineStr">
-        <is>
-          <t>AL25REG</t>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>AL55REG</t>
         </is>
       </c>
     </row>
@@ -2412,51 +2752,63 @@
         </is>
       </c>
       <c r="G30" t="n">
+        <v>367</v>
+      </c>
+      <c r="H30" t="n">
+        <v>10</v>
+      </c>
+      <c r="I30" t="n">
+        <v>5</v>
+      </c>
+      <c r="J30" t="n">
+        <v>5</v>
+      </c>
+      <c r="K30" t="n">
         <v>232</v>
       </c>
-      <c r="H30" t="n">
+      <c r="L30" t="n">
         <v>0.65</v>
       </c>
-      <c r="I30" t="n">
+      <c r="M30" t="n">
         <v>135.72</v>
       </c>
-      <c r="J30" t="n">
+      <c r="N30" t="n">
         <v>123.505</v>
       </c>
-      <c r="K30" t="n">
+      <c r="O30" t="n">
         <v>86.453</v>
       </c>
-      <c r="L30" t="n">
+      <c r="P30" t="n">
         <v>98.804</v>
       </c>
-      <c r="M30" t="inlineStr">
+      <c r="Q30" t="inlineStr">
         <is>
           <t>South Korea-KR</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr">
+      <c r="R30" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 26</t>
         </is>
       </c>
-      <c r="O30" t="inlineStr">
+      <c r="S30" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P30" t="inlineStr">
+      <c r="T30" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-26</t>
         </is>
       </c>
-      <c r="Q30" t="inlineStr">
+      <c r="U30" t="inlineStr">
         <is>
           <t>AL26 0AA</t>
         </is>
       </c>
-      <c r="R30" t="inlineStr">
-        <is>
-          <t>AL26REG</t>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>AL66REG</t>
         </is>
       </c>
     </row>
@@ -2484,48 +2836,60 @@
         </is>
       </c>
       <c r="G31" t="n">
+        <v>254</v>
+      </c>
+      <c r="H31" t="n">
+        <v>10</v>
+      </c>
+      <c r="I31" t="n">
+        <v>5</v>
+      </c>
+      <c r="J31" t="n">
+        <v>5</v>
+      </c>
+      <c r="K31" t="n">
         <v>239</v>
       </c>
-      <c r="H31" t="n">
+      <c r="L31" t="n">
         <v>0.975</v>
       </c>
-      <c r="I31" t="n">
+      <c r="M31" t="n">
         <v>209.722</v>
       </c>
-      <c r="J31" t="n">
+      <c r="N31" t="n">
         <v>192.944</v>
       </c>
-      <c r="K31" t="n">
+      <c r="O31" t="n">
         <v>189.085</v>
       </c>
-      <c r="M31" t="inlineStr">
+      <c r="Q31" t="inlineStr">
         <is>
           <t>Italy-IT</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr">
+      <c r="R31" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 27</t>
         </is>
       </c>
-      <c r="O31" t="inlineStr">
+      <c r="S31" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P31" t="inlineStr">
+      <c r="T31" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-27</t>
         </is>
       </c>
-      <c r="Q31" t="inlineStr">
+      <c r="U31" t="inlineStr">
         <is>
           <t>AL27 0AA</t>
         </is>
       </c>
-      <c r="R31" t="inlineStr">
-        <is>
-          <t>AL27REG</t>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>NOTAPLATE</t>
         </is>
       </c>
     </row>
@@ -2553,48 +2917,60 @@
         </is>
       </c>
       <c r="G32" t="n">
+        <v>261</v>
+      </c>
+      <c r="H32" t="n">
+        <v>10</v>
+      </c>
+      <c r="I32" t="n">
+        <v>5</v>
+      </c>
+      <c r="J32" t="n">
+        <v>5</v>
+      </c>
+      <c r="K32" t="n">
         <v>246</v>
       </c>
-      <c r="H32" t="n">
+      <c r="L32" t="n">
         <v>0.875</v>
       </c>
-      <c r="I32" t="n">
+      <c r="M32" t="n">
         <v>193.725</v>
       </c>
-      <c r="J32" t="n">
+      <c r="N32" t="n">
         <v>180.164</v>
       </c>
-      <c r="K32" t="n">
+      <c r="O32" t="n">
         <v>165.751</v>
       </c>
-      <c r="M32" t="inlineStr">
+      <c r="Q32" t="inlineStr">
         <is>
           <t>Germany-DE</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>E-ACC10001AL Reprocessor 28</t>
-        </is>
-      </c>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="P32" t="inlineStr">
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Global Reprocessing Ltd</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-28</t>
         </is>
       </c>
-      <c r="Q32" t="inlineStr">
+      <c r="U32" t="inlineStr">
         <is>
           <t>AL28 0AA</t>
         </is>
       </c>
-      <c r="R32" t="inlineStr">
-        <is>
-          <t>AL28REG</t>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>AL88REG</t>
         </is>
       </c>
     </row>
@@ -2622,48 +2998,60 @@
         </is>
       </c>
       <c r="G33" t="n">
+        <v>268</v>
+      </c>
+      <c r="H33" t="n">
+        <v>10</v>
+      </c>
+      <c r="I33" t="n">
+        <v>5</v>
+      </c>
+      <c r="J33" t="n">
+        <v>5</v>
+      </c>
+      <c r="K33" t="n">
         <v>253</v>
       </c>
-      <c r="H33" t="n">
+      <c r="L33" t="n">
         <v>0.65</v>
       </c>
-      <c r="I33" t="n">
+      <c r="M33" t="n">
         <v>148.005</v>
       </c>
-      <c r="J33" t="n">
+      <c r="N33" t="n">
         <v>139.125</v>
       </c>
-      <c r="K33" t="n">
+      <c r="O33" t="n">
         <v>130.778</v>
       </c>
-      <c r="M33" t="inlineStr">
+      <c r="Q33" t="inlineStr">
         <is>
           <t>Spain-ES</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>E-ACC10001AL Reprocessor 29</t>
-        </is>
-      </c>
-      <c r="O33" t="inlineStr">
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>Global Reprocessing Ltd</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P33" t="inlineStr">
+      <c r="T33" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-29</t>
         </is>
       </c>
-      <c r="Q33" t="inlineStr">
+      <c r="U33" t="inlineStr">
         <is>
           <t>AL29 0AA</t>
         </is>
       </c>
-      <c r="R33" t="inlineStr">
-        <is>
-          <t>AL29REG</t>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>AL99REG</t>
         </is>
       </c>
     </row>
@@ -2691,51 +3079,63 @@
         </is>
       </c>
       <c r="G34" t="n">
+        <v>275</v>
+      </c>
+      <c r="H34" t="n">
+        <v>10</v>
+      </c>
+      <c r="I34" t="n">
+        <v>5</v>
+      </c>
+      <c r="J34" t="n">
+        <v>5</v>
+      </c>
+      <c r="K34" t="n">
         <v>260</v>
       </c>
-      <c r="H34" t="n">
+      <c r="L34" t="n">
         <v>0.975</v>
       </c>
-      <c r="I34" t="n">
+      <c r="M34" t="n">
         <v>228.15</v>
       </c>
-      <c r="J34" t="n">
+      <c r="N34" t="n">
         <v>205.335</v>
       </c>
-      <c r="K34" t="n">
+      <c r="O34" t="n">
         <v>143.734</v>
       </c>
-      <c r="L34" t="n">
+      <c r="P34" t="n">
         <v>164.268</v>
       </c>
-      <c r="M34" t="inlineStr">
+      <c r="Q34" t="inlineStr">
         <is>
           <t>Netherlands-NL</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>E-ACC10001AL Reprocessor 30</t>
-        </is>
-      </c>
-      <c r="O34" t="inlineStr">
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>Global Reprocessing Ltd</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P34" t="inlineStr">
+      <c r="T34" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-30</t>
         </is>
       </c>
-      <c r="Q34" t="inlineStr">
+      <c r="U34" t="inlineStr">
         <is>
           <t>AL30 0AA</t>
         </is>
       </c>
-      <c r="R34" t="inlineStr">
-        <is>
-          <t>AL30REG</t>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>AL00REG</t>
         </is>
       </c>
     </row>
@@ -2763,51 +3163,63 @@
         </is>
       </c>
       <c r="G35" t="n">
+        <v>282</v>
+      </c>
+      <c r="H35" t="n">
+        <v>10</v>
+      </c>
+      <c r="I35" t="n">
+        <v>5</v>
+      </c>
+      <c r="J35" t="n">
+        <v>5</v>
+      </c>
+      <c r="K35" t="n">
         <v>267</v>
       </c>
-      <c r="H35" t="n">
+      <c r="L35" t="n">
         <v>0.875</v>
       </c>
-      <c r="I35" t="n">
+      <c r="M35" t="n">
         <v>210.263</v>
       </c>
-      <c r="J35" t="n">
+      <c r="N35" t="n">
         <v>191.339</v>
       </c>
-      <c r="K35" t="n">
+      <c r="O35" t="n">
         <v>133.937</v>
       </c>
-      <c r="L35" t="n">
+      <c r="P35" t="n">
         <v>153.071</v>
       </c>
-      <c r="M35" t="inlineStr">
+      <c r="Q35" t="inlineStr">
         <is>
           <t>India-IN</t>
         </is>
       </c>
-      <c r="N35" t="inlineStr">
+      <c r="R35" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 31</t>
         </is>
       </c>
-      <c r="O35" t="inlineStr">
+      <c r="S35" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P35" t="inlineStr">
+      <c r="T35" t="inlineStr">
         <is>
           <t>Shared Metals Recovery Ltd</t>
         </is>
       </c>
-      <c r="Q35" t="inlineStr">
+      <c r="U35" t="inlineStr">
         <is>
           <t>LS1 4AB</t>
         </is>
       </c>
-      <c r="R35" t="inlineStr">
-        <is>
-          <t>AL31REG</t>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>AL11REG</t>
         </is>
       </c>
     </row>
@@ -2835,48 +3247,60 @@
         </is>
       </c>
       <c r="G36" t="n">
+        <v>289</v>
+      </c>
+      <c r="H36" t="n">
+        <v>10</v>
+      </c>
+      <c r="I36" t="n">
+        <v>5</v>
+      </c>
+      <c r="J36" t="n">
+        <v>5</v>
+      </c>
+      <c r="K36" t="n">
         <v>274</v>
       </c>
-      <c r="H36" t="n">
+      <c r="L36" t="n">
         <v>0.65</v>
       </c>
-      <c r="I36" t="n">
+      <c r="M36" t="n">
         <v>160.29</v>
       </c>
-      <c r="J36" t="n">
+      <c r="N36" t="n">
         <v>147.467</v>
       </c>
-      <c r="K36" t="n">
+      <c r="O36" t="n">
         <v>135.67</v>
       </c>
-      <c r="M36" t="inlineStr">
+      <c r="Q36" t="inlineStr">
         <is>
           <t>Turkey-TR</t>
         </is>
       </c>
-      <c r="N36" t="inlineStr">
+      <c r="R36" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 32</t>
         </is>
       </c>
-      <c r="O36" t="inlineStr">
+      <c r="S36" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P36" t="inlineStr">
+      <c r="T36" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-32</t>
         </is>
       </c>
-      <c r="Q36" t="inlineStr">
+      <c r="U36" t="inlineStr">
         <is>
           <t>AL32 0AA</t>
         </is>
       </c>
-      <c r="R36" t="inlineStr">
-        <is>
-          <t>AL32REG</t>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>AL22REG</t>
         </is>
       </c>
     </row>
@@ -2904,46 +3328,58 @@
         </is>
       </c>
       <c r="G37" t="n">
+        <v>296</v>
+      </c>
+      <c r="H37" t="n">
+        <v>10</v>
+      </c>
+      <c r="I37" t="n">
+        <v>5</v>
+      </c>
+      <c r="J37" t="n">
+        <v>5</v>
+      </c>
+      <c r="K37" t="n">
         <v>281</v>
       </c>
-      <c r="H37" t="n">
+      <c r="L37" t="n">
         <v>0.975</v>
       </c>
-      <c r="I37" t="n">
+      <c r="M37" t="n">
         <v>246.577</v>
       </c>
-      <c r="J37" t="n">
+      <c r="N37" t="n">
         <v>229.317</v>
       </c>
-      <c r="K37" t="n">
+      <c r="O37" t="n">
         <v>215.558</v>
       </c>
-      <c r="M37" t="inlineStr">
+      <c r="Q37" t="inlineStr">
         <is>
           <t>South Korea-KR</t>
         </is>
       </c>
-      <c r="N37" t="inlineStr">
+      <c r="R37" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 33</t>
         </is>
       </c>
-      <c r="O37" t="inlineStr">
+      <c r="S37" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P37" t="inlineStr">
+      <c r="T37" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-33</t>
         </is>
       </c>
-      <c r="Q37" t="inlineStr">
+      <c r="U37" t="inlineStr">
         <is>
           <t>AL33 0AA</t>
         </is>
       </c>
-      <c r="R37" t="inlineStr">
+      <c r="V37" t="inlineStr">
         <is>
           <t>AL33REG</t>
         </is>
@@ -2973,48 +3409,60 @@
         </is>
       </c>
       <c r="G38" t="n">
+        <v>303</v>
+      </c>
+      <c r="H38" t="n">
+        <v>10</v>
+      </c>
+      <c r="I38" t="n">
+        <v>5</v>
+      </c>
+      <c r="J38" t="n">
+        <v>5</v>
+      </c>
+      <c r="K38" t="n">
         <v>288</v>
       </c>
-      <c r="H38" t="n">
+      <c r="L38" t="n">
         <v>0.875</v>
       </c>
-      <c r="I38" t="n">
+      <c r="M38" t="n">
         <v>226.8</v>
       </c>
-      <c r="J38" t="n">
+      <c r="N38" t="n">
         <v>213.192</v>
       </c>
-      <c r="K38" t="n">
+      <c r="O38" t="n">
         <v>204.664</v>
       </c>
-      <c r="M38" t="inlineStr">
+      <c r="Q38" t="inlineStr">
         <is>
           <t>Italy-IT</t>
         </is>
       </c>
-      <c r="N38" t="inlineStr">
+      <c r="R38" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 34</t>
         </is>
       </c>
-      <c r="O38" t="inlineStr">
+      <c r="S38" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P38" t="inlineStr">
+      <c r="T38" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-34</t>
         </is>
       </c>
-      <c r="Q38" t="inlineStr">
+      <c r="U38" t="inlineStr">
         <is>
           <t>AL34 0AA</t>
         </is>
       </c>
-      <c r="R38" t="inlineStr">
-        <is>
-          <t>AL34REG</t>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>AL44REG</t>
         </is>
       </c>
     </row>
@@ -3042,51 +3490,63 @@
         </is>
       </c>
       <c r="G39" t="n">
+        <v>310</v>
+      </c>
+      <c r="H39" t="n">
+        <v>10</v>
+      </c>
+      <c r="I39" t="n">
+        <v>5</v>
+      </c>
+      <c r="J39" t="n">
+        <v>5</v>
+      </c>
+      <c r="K39" t="n">
         <v>295</v>
       </c>
-      <c r="H39" t="n">
+      <c r="L39" t="n">
         <v>0.65</v>
       </c>
-      <c r="I39" t="n">
+      <c r="M39" t="n">
         <v>172.575</v>
       </c>
-      <c r="J39" t="n">
+      <c r="N39" t="n">
         <v>155.317</v>
       </c>
-      <c r="K39" t="n">
+      <c r="O39" t="n">
         <v>108.722</v>
       </c>
-      <c r="L39" t="n">
+      <c r="P39" t="n">
         <v>124.254</v>
       </c>
-      <c r="M39" t="inlineStr">
+      <c r="Q39" t="inlineStr">
         <is>
           <t>Germany-DE</t>
         </is>
       </c>
-      <c r="N39" t="inlineStr">
+      <c r="R39" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 35</t>
         </is>
       </c>
-      <c r="O39" t="inlineStr">
+      <c r="S39" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P39" t="inlineStr">
+      <c r="T39" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-35</t>
         </is>
       </c>
-      <c r="Q39" t="inlineStr">
+      <c r="U39" t="inlineStr">
         <is>
           <t>AL35 0AA</t>
         </is>
       </c>
-      <c r="R39" t="inlineStr">
-        <is>
-          <t>AL35REG</t>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>AL55REG</t>
         </is>
       </c>
     </row>
@@ -3114,51 +3574,63 @@
         </is>
       </c>
       <c r="G40" t="n">
+        <v>317</v>
+      </c>
+      <c r="H40" t="n">
+        <v>10</v>
+      </c>
+      <c r="I40" t="n">
+        <v>5</v>
+      </c>
+      <c r="J40" t="n">
+        <v>5</v>
+      </c>
+      <c r="K40" t="n">
         <v>302</v>
       </c>
-      <c r="H40" t="n">
+      <c r="L40" t="n">
         <v>0.975</v>
       </c>
-      <c r="I40" t="n">
+      <c r="M40" t="n">
         <v>265.005</v>
       </c>
-      <c r="J40" t="n">
+      <c r="N40" t="n">
         <v>241.155</v>
       </c>
-      <c r="K40" t="n">
+      <c r="O40" t="n">
         <v>168.808</v>
       </c>
-      <c r="L40" t="n">
+      <c r="P40" t="n">
         <v>192.924</v>
       </c>
-      <c r="M40" t="inlineStr">
+      <c r="Q40" t="inlineStr">
         <is>
           <t>Spain-ES</t>
         </is>
       </c>
-      <c r="N40" t="inlineStr">
+      <c r="R40" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 36</t>
         </is>
       </c>
-      <c r="O40" t="inlineStr">
+      <c r="S40" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P40" t="inlineStr">
+      <c r="T40" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-36</t>
         </is>
       </c>
-      <c r="Q40" t="inlineStr">
+      <c r="U40" t="inlineStr">
         <is>
           <t>AL36 0AA</t>
         </is>
       </c>
-      <c r="R40" t="inlineStr">
-        <is>
-          <t>AL36REG</t>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>AL66REG</t>
         </is>
       </c>
     </row>
@@ -3186,48 +3658,60 @@
         </is>
       </c>
       <c r="G41" t="n">
+        <v>324</v>
+      </c>
+      <c r="H41" t="n">
+        <v>10</v>
+      </c>
+      <c r="I41" t="n">
+        <v>5</v>
+      </c>
+      <c r="J41" t="n">
+        <v>5</v>
+      </c>
+      <c r="K41" t="n">
         <v>309</v>
       </c>
-      <c r="H41" t="n">
+      <c r="L41" t="n">
         <v>0.875</v>
       </c>
-      <c r="I41" t="n">
+      <c r="M41" t="n">
         <v>243.338</v>
       </c>
-      <c r="J41" t="n">
+      <c r="N41" t="n">
         <v>223.871</v>
       </c>
-      <c r="K41" t="n">
+      <c r="O41" t="n">
         <v>210.439</v>
       </c>
-      <c r="M41" t="inlineStr">
+      <c r="Q41" t="inlineStr">
         <is>
           <t>Netherlands-NL</t>
         </is>
       </c>
-      <c r="N41" t="inlineStr">
+      <c r="R41" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 37</t>
         </is>
       </c>
-      <c r="O41" t="inlineStr">
+      <c r="S41" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P41" t="inlineStr">
+      <c r="T41" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-37</t>
         </is>
       </c>
-      <c r="Q41" t="inlineStr">
+      <c r="U41" t="inlineStr">
         <is>
           <t>AL37 0AA</t>
         </is>
       </c>
-      <c r="R41" t="inlineStr">
-        <is>
-          <t>AL37REG</t>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>AL77REG</t>
         </is>
       </c>
     </row>
@@ -3255,48 +3739,60 @@
         </is>
       </c>
       <c r="G42" t="n">
+        <v>331</v>
+      </c>
+      <c r="H42" t="n">
+        <v>10</v>
+      </c>
+      <c r="I42" t="n">
+        <v>5</v>
+      </c>
+      <c r="J42" t="n">
+        <v>5</v>
+      </c>
+      <c r="K42" t="n">
         <v>316</v>
       </c>
-      <c r="H42" t="n">
+      <c r="L42" t="n">
         <v>0.65</v>
       </c>
-      <c r="I42" t="n">
+      <c r="M42" t="n">
         <v>184.86</v>
       </c>
-      <c r="J42" t="n">
+      <c r="N42" t="n">
         <v>171.92</v>
       </c>
-      <c r="K42" t="n">
+      <c r="O42" t="n">
         <v>165.043</v>
       </c>
-      <c r="M42" t="inlineStr">
+      <c r="Q42" t="inlineStr">
         <is>
           <t>India-IN</t>
         </is>
       </c>
-      <c r="N42" t="inlineStr">
+      <c r="R42" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 38</t>
         </is>
       </c>
-      <c r="O42" t="inlineStr">
+      <c r="S42" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P42" t="inlineStr">
+      <c r="T42" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-38</t>
         </is>
       </c>
-      <c r="Q42" t="inlineStr">
+      <c r="U42" t="inlineStr">
         <is>
           <t>AL38 0AA</t>
         </is>
       </c>
-      <c r="R42" t="inlineStr">
-        <is>
-          <t>AL38REG</t>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>AL88REG</t>
         </is>
       </c>
     </row>
@@ -3324,48 +3820,60 @@
         </is>
       </c>
       <c r="G43" t="n">
+        <v>338</v>
+      </c>
+      <c r="H43" t="n">
+        <v>10</v>
+      </c>
+      <c r="I43" t="n">
+        <v>5</v>
+      </c>
+      <c r="J43" t="n">
+        <v>5</v>
+      </c>
+      <c r="K43" t="n">
         <v>323</v>
       </c>
-      <c r="H43" t="n">
+      <c r="L43" t="n">
         <v>0.975</v>
       </c>
-      <c r="I43" t="n">
+      <c r="M43" t="n">
         <v>283.433</v>
       </c>
-      <c r="J43" t="n">
+      <c r="N43" t="n">
         <v>266.427</v>
       </c>
-      <c r="K43" t="n">
+      <c r="O43" t="n">
         <v>261.098</v>
       </c>
-      <c r="M43" t="inlineStr">
+      <c r="Q43" t="inlineStr">
         <is>
           <t>Turkey-TR</t>
         </is>
       </c>
-      <c r="N43" t="inlineStr">
+      <c r="R43" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 39</t>
         </is>
       </c>
-      <c r="O43" t="inlineStr">
+      <c r="S43" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P43" t="inlineStr">
+      <c r="T43" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-39</t>
         </is>
       </c>
-      <c r="Q43" t="inlineStr">
+      <c r="U43" t="inlineStr">
         <is>
           <t>AL39 0AA</t>
         </is>
       </c>
-      <c r="R43" t="inlineStr">
-        <is>
-          <t>AL39REG</t>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>AL99REG</t>
         </is>
       </c>
     </row>
@@ -3393,51 +3901,63 @@
         </is>
       </c>
       <c r="G44" t="n">
+        <v>345</v>
+      </c>
+      <c r="H44" t="n">
+        <v>10</v>
+      </c>
+      <c r="I44" t="n">
+        <v>5</v>
+      </c>
+      <c r="J44" t="n">
+        <v>5</v>
+      </c>
+      <c r="K44" t="n">
         <v>330</v>
       </c>
-      <c r="H44" t="n">
+      <c r="L44" t="n">
         <v>0.875</v>
       </c>
-      <c r="I44" t="n">
+      <c r="M44" t="n">
         <v>259.875</v>
       </c>
-      <c r="J44" t="n">
+      <c r="N44" t="n">
         <v>233.888</v>
       </c>
-      <c r="K44" t="n">
+      <c r="O44" t="n">
         <v>163.722</v>
       </c>
-      <c r="L44" t="n">
+      <c r="P44" t="n">
         <v>187.11</v>
       </c>
-      <c r="M44" t="inlineStr">
+      <c r="Q44" t="inlineStr">
         <is>
           <t>South Korea-KR</t>
         </is>
       </c>
-      <c r="N44" t="inlineStr">
+      <c r="R44" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 40</t>
         </is>
       </c>
-      <c r="O44" t="inlineStr">
+      <c r="S44" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P44" t="inlineStr">
+      <c r="T44" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-40</t>
         </is>
       </c>
-      <c r="Q44" t="inlineStr">
+      <c r="U44" t="inlineStr">
         <is>
           <t>AL40 0AA</t>
         </is>
       </c>
-      <c r="R44" t="inlineStr">
-        <is>
-          <t>AL40REG</t>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>AL00REG</t>
         </is>
       </c>
     </row>
@@ -3465,51 +3985,63 @@
         </is>
       </c>
       <c r="G45" t="n">
+        <v>352</v>
+      </c>
+      <c r="H45" t="n">
+        <v>10</v>
+      </c>
+      <c r="I45" t="n">
+        <v>5</v>
+      </c>
+      <c r="J45" t="n">
+        <v>5</v>
+      </c>
+      <c r="K45" t="n">
         <v>337</v>
       </c>
-      <c r="H45" t="n">
+      <c r="L45" t="n">
         <v>0.65</v>
       </c>
-      <c r="I45" t="n">
+      <c r="M45" t="n">
         <v>197.145</v>
       </c>
-      <c r="J45" t="n">
+      <c r="N45" t="n">
         <v>179.402</v>
       </c>
-      <c r="K45" t="n">
+      <c r="O45" t="n">
         <v>125.581</v>
       </c>
-      <c r="L45" t="n">
+      <c r="P45" t="n">
         <v>143.522</v>
       </c>
-      <c r="M45" t="inlineStr">
+      <c r="Q45" t="inlineStr">
         <is>
           <t>Italy-IT</t>
         </is>
       </c>
-      <c r="N45" t="inlineStr">
+      <c r="R45" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 41</t>
         </is>
       </c>
-      <c r="O45" t="inlineStr">
+      <c r="S45" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P45" t="inlineStr">
+      <c r="T45" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-41</t>
         </is>
       </c>
-      <c r="Q45" t="inlineStr">
+      <c r="U45" t="inlineStr">
         <is>
           <t>AL41 0AA</t>
         </is>
       </c>
-      <c r="R45" t="inlineStr">
-        <is>
-          <t>AL41REG</t>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>AL11REG</t>
         </is>
       </c>
     </row>
@@ -3537,48 +4069,60 @@
         </is>
       </c>
       <c r="G46" t="n">
+        <v>359</v>
+      </c>
+      <c r="H46" t="n">
+        <v>10</v>
+      </c>
+      <c r="I46" t="n">
+        <v>5</v>
+      </c>
+      <c r="J46" t="n">
+        <v>5</v>
+      </c>
+      <c r="K46" t="n">
         <v>344</v>
       </c>
-      <c r="H46" t="n">
+      <c r="L46" t="n">
         <v>0.975</v>
       </c>
-      <c r="I46" t="n">
+      <c r="M46" t="n">
         <v>301.86</v>
       </c>
-      <c r="J46" t="n">
+      <c r="N46" t="n">
         <v>277.711</v>
       </c>
-      <c r="K46" t="n">
+      <c r="O46" t="n">
         <v>266.603</v>
       </c>
-      <c r="M46" t="inlineStr">
+      <c r="Q46" t="inlineStr">
         <is>
           <t>Germany-DE</t>
         </is>
       </c>
-      <c r="N46" t="inlineStr">
+      <c r="R46" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 42</t>
         </is>
       </c>
-      <c r="O46" t="inlineStr">
+      <c r="S46" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P46" t="inlineStr">
+      <c r="T46" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-42</t>
         </is>
       </c>
-      <c r="Q46" t="inlineStr">
+      <c r="U46" t="inlineStr">
         <is>
           <t>AL42 0AA</t>
         </is>
       </c>
-      <c r="R46" t="inlineStr">
-        <is>
-          <t>AL42REG</t>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>AL22REG</t>
         </is>
       </c>
     </row>
@@ -3606,48 +4150,60 @@
         </is>
       </c>
       <c r="G47" t="n">
+        <v>366</v>
+      </c>
+      <c r="H47" t="n">
+        <v>10</v>
+      </c>
+      <c r="I47" t="n">
+        <v>5</v>
+      </c>
+      <c r="J47" t="n">
+        <v>5</v>
+      </c>
+      <c r="K47" t="n">
         <v>351</v>
       </c>
-      <c r="H47" t="n">
+      <c r="L47" t="n">
         <v>0.875</v>
       </c>
-      <c r="I47" t="n">
+      <c r="M47" t="n">
         <v>276.413</v>
       </c>
-      <c r="J47" t="n">
+      <c r="N47" t="n">
         <v>257.064</v>
       </c>
-      <c r="K47" t="n">
+      <c r="O47" t="n">
         <v>251.923</v>
       </c>
-      <c r="M47" t="inlineStr">
+      <c r="Q47" t="inlineStr">
         <is>
           <t>Spain-ES</t>
         </is>
       </c>
-      <c r="N47" t="inlineStr">
+      <c r="R47" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 43</t>
         </is>
       </c>
-      <c r="O47" t="inlineStr">
+      <c r="S47" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P47" t="inlineStr">
+      <c r="T47" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-43</t>
         </is>
       </c>
-      <c r="Q47" t="inlineStr">
+      <c r="U47" t="inlineStr">
         <is>
           <t>AL43 0AA</t>
         </is>
       </c>
-      <c r="R47" t="inlineStr">
-        <is>
-          <t>AL43REG</t>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>AL33REG</t>
         </is>
       </c>
     </row>
@@ -3675,46 +4231,58 @@
         </is>
       </c>
       <c r="G48" t="n">
+        <v>373</v>
+      </c>
+      <c r="H48" t="n">
+        <v>10</v>
+      </c>
+      <c r="I48" t="n">
+        <v>5</v>
+      </c>
+      <c r="J48" t="n">
+        <v>5</v>
+      </c>
+      <c r="K48" t="n">
         <v>358</v>
       </c>
-      <c r="H48" t="n">
+      <c r="L48" t="n">
         <v>0.65</v>
       </c>
-      <c r="I48" t="n">
+      <c r="M48" t="n">
         <v>209.43</v>
       </c>
-      <c r="J48" t="n">
+      <c r="N48" t="n">
         <v>196.864</v>
       </c>
-      <c r="K48" t="n">
+      <c r="O48" t="n">
         <v>181.115</v>
       </c>
-      <c r="M48" t="inlineStr">
+      <c r="Q48" t="inlineStr">
         <is>
           <t>Netherlands-NL</t>
         </is>
       </c>
-      <c r="N48" t="inlineStr">
+      <c r="R48" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 44</t>
         </is>
       </c>
-      <c r="O48" t="inlineStr">
+      <c r="S48" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P48" t="inlineStr">
+      <c r="T48" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-44</t>
         </is>
       </c>
-      <c r="Q48" t="inlineStr">
+      <c r="U48" t="inlineStr">
         <is>
           <t>AL44 0AA</t>
         </is>
       </c>
-      <c r="R48" t="inlineStr">
+      <c r="V48" t="inlineStr">
         <is>
           <t>AL44REG</t>
         </is>
@@ -3744,51 +4312,63 @@
         </is>
       </c>
       <c r="G49" t="n">
+        <v>380</v>
+      </c>
+      <c r="H49" t="n">
+        <v>10</v>
+      </c>
+      <c r="I49" t="n">
+        <v>5</v>
+      </c>
+      <c r="J49" t="n">
+        <v>5</v>
+      </c>
+      <c r="K49" t="n">
         <v>365</v>
       </c>
-      <c r="H49" t="n">
+      <c r="L49" t="n">
         <v>0.975</v>
       </c>
-      <c r="I49" t="n">
+      <c r="M49" t="n">
         <v>320.288</v>
       </c>
-      <c r="J49" t="n">
+      <c r="N49" t="n">
         <v>288.259</v>
       </c>
-      <c r="K49" t="n">
+      <c r="O49" t="n">
         <v>201.781</v>
       </c>
-      <c r="L49" t="n">
+      <c r="P49" t="n">
         <v>230.607</v>
       </c>
-      <c r="M49" t="inlineStr">
+      <c r="Q49" t="inlineStr">
         <is>
           <t>India-IN</t>
         </is>
       </c>
-      <c r="N49" t="inlineStr">
+      <c r="R49" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 45</t>
         </is>
       </c>
-      <c r="O49" t="inlineStr">
+      <c r="S49" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P49" t="inlineStr">
+      <c r="T49" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-45</t>
         </is>
       </c>
-      <c r="Q49" t="inlineStr">
+      <c r="U49" t="inlineStr">
         <is>
           <t>AL45 0AA</t>
         </is>
       </c>
-      <c r="R49" t="inlineStr">
-        <is>
-          <t>AL45REG</t>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>AL55REG</t>
         </is>
       </c>
     </row>
@@ -3816,51 +4396,63 @@
         </is>
       </c>
       <c r="G50" t="n">
+        <v>387</v>
+      </c>
+      <c r="H50" t="n">
+        <v>10</v>
+      </c>
+      <c r="I50" t="n">
+        <v>5</v>
+      </c>
+      <c r="J50" t="n">
+        <v>5</v>
+      </c>
+      <c r="K50" t="n">
         <v>372</v>
       </c>
-      <c r="H50" t="n">
+      <c r="L50" t="n">
         <v>0.875</v>
       </c>
-      <c r="I50" t="n">
+      <c r="M50" t="n">
         <v>292.95</v>
       </c>
-      <c r="J50" t="n">
+      <c r="N50" t="n">
         <v>266.584</v>
       </c>
-      <c r="K50" t="n">
+      <c r="O50" t="n">
         <v>186.609</v>
       </c>
-      <c r="L50" t="n">
+      <c r="P50" t="n">
         <v>213.267</v>
       </c>
-      <c r="M50" t="inlineStr">
+      <c r="Q50" t="inlineStr">
         <is>
           <t>Turkey-TR</t>
         </is>
       </c>
-      <c r="N50" t="inlineStr">
+      <c r="R50" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 46</t>
         </is>
       </c>
-      <c r="O50" t="inlineStr">
+      <c r="S50" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P50" t="inlineStr">
+      <c r="T50" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-46</t>
         </is>
       </c>
-      <c r="Q50" t="inlineStr">
+      <c r="U50" t="inlineStr">
         <is>
           <t>AL46 0AA</t>
         </is>
       </c>
-      <c r="R50" t="inlineStr">
-        <is>
-          <t>AL46REG</t>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>AL66REG</t>
         </is>
       </c>
     </row>
@@ -3888,48 +4480,60 @@
         </is>
       </c>
       <c r="G51" t="n">
+        <v>394</v>
+      </c>
+      <c r="H51" t="n">
+        <v>10</v>
+      </c>
+      <c r="I51" t="n">
+        <v>5</v>
+      </c>
+      <c r="J51" t="n">
+        <v>5</v>
+      </c>
+      <c r="K51" t="n">
         <v>379</v>
       </c>
-      <c r="H51" t="n">
+      <c r="L51" t="n">
         <v>0.65</v>
       </c>
-      <c r="I51" t="n">
+      <c r="M51" t="n">
         <v>221.715</v>
       </c>
-      <c r="J51" t="n">
+      <c r="N51" t="n">
         <v>203.978</v>
       </c>
-      <c r="K51" t="n">
+      <c r="O51" t="n">
         <v>199.898</v>
       </c>
-      <c r="M51" t="inlineStr">
+      <c r="Q51" t="inlineStr">
         <is>
           <t>South Korea-KR</t>
         </is>
       </c>
-      <c r="N51" t="inlineStr">
+      <c r="R51" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 47</t>
         </is>
       </c>
-      <c r="O51" t="inlineStr">
+      <c r="S51" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P51" t="inlineStr">
+      <c r="T51" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-47</t>
         </is>
       </c>
-      <c r="Q51" t="inlineStr">
+      <c r="U51" t="inlineStr">
         <is>
           <t>AL47 0AA</t>
         </is>
       </c>
-      <c r="R51" t="inlineStr">
-        <is>
-          <t>AL47REG</t>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>AL77REG</t>
         </is>
       </c>
     </row>
@@ -3957,48 +4561,60 @@
         </is>
       </c>
       <c r="G52" t="n">
+        <v>401</v>
+      </c>
+      <c r="H52" t="n">
+        <v>10</v>
+      </c>
+      <c r="I52" t="n">
+        <v>5</v>
+      </c>
+      <c r="J52" t="n">
+        <v>5</v>
+      </c>
+      <c r="K52" t="n">
         <v>386</v>
       </c>
-      <c r="H52" t="n">
+      <c r="L52" t="n">
         <v>0.975</v>
       </c>
-      <c r="I52" t="n">
+      <c r="M52" t="n">
         <v>338.715</v>
       </c>
-      <c r="J52" t="n">
+      <c r="N52" t="n">
         <v>315.005</v>
       </c>
-      <c r="K52" t="n">
+      <c r="O52" t="n">
         <v>289.805</v>
       </c>
-      <c r="M52" t="inlineStr">
+      <c r="Q52" t="inlineStr">
         <is>
           <t>Italy-IT</t>
         </is>
       </c>
-      <c r="N52" t="inlineStr">
+      <c r="R52" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 48</t>
         </is>
       </c>
-      <c r="O52" t="inlineStr">
+      <c r="S52" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P52" t="inlineStr">
+      <c r="T52" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-48</t>
         </is>
       </c>
-      <c r="Q52" t="inlineStr">
+      <c r="U52" t="inlineStr">
         <is>
           <t>AL48 0AA</t>
         </is>
       </c>
-      <c r="R52" t="inlineStr">
-        <is>
-          <t>AL48REG</t>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>AL88REG</t>
         </is>
       </c>
     </row>
@@ -4026,48 +4642,60 @@
         </is>
       </c>
       <c r="G53" t="n">
+        <v>408</v>
+      </c>
+      <c r="H53" t="n">
+        <v>10</v>
+      </c>
+      <c r="I53" t="n">
+        <v>5</v>
+      </c>
+      <c r="J53" t="n">
+        <v>5</v>
+      </c>
+      <c r="K53" t="n">
         <v>393</v>
       </c>
-      <c r="H53" t="n">
+      <c r="L53" t="n">
         <v>0.875</v>
       </c>
-      <c r="I53" t="n">
+      <c r="M53" t="n">
         <v>309.488</v>
       </c>
-      <c r="J53" t="n">
+      <c r="N53" t="n">
         <v>290.919</v>
       </c>
-      <c r="K53" t="n">
+      <c r="O53" t="n">
         <v>273.464</v>
       </c>
-      <c r="M53" t="inlineStr">
+      <c r="Q53" t="inlineStr">
         <is>
           <t>Germany-DE</t>
         </is>
       </c>
-      <c r="N53" t="inlineStr">
+      <c r="R53" t="inlineStr">
         <is>
           <t>E-ACC10001AL Reprocessor 49</t>
         </is>
       </c>
-      <c r="O53" t="inlineStr">
+      <c r="S53" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P53" t="inlineStr">
+      <c r="T53" t="inlineStr">
         <is>
           <t>Supplier E-ACC10001AL-49</t>
         </is>
       </c>
-      <c r="Q53" t="inlineStr">
+      <c r="U53" t="inlineStr">
         <is>
           <t>AL49 0AA</t>
         </is>
       </c>
-      <c r="R53" t="inlineStr">
-        <is>
-          <t>AL49REG</t>
+      <c r="V53" t="inlineStr">
+        <is>
+          <t>AL99REG</t>
         </is>
       </c>
     </row>

</xml_diff>